<commit_message>
Update : Insert DAPODIK code in Region Page
</commit_message>
<xml_diff>
--- a/_Page/Wilayah/Template-Wilayah.xlsx
+++ b/_Page/Wilayah/Template-Wilayah.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RTG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\rtgadd\_Page\Wilayah\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{02462A3A-84A2-4B8D-AE1F-0D628DFBF850}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790183AD-E24B-459F-94E7-B637AF32985B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B4ACC4A9-CB3D-47B0-9317-38B520C4B3B5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="37">
   <si>
     <t>15</t>
   </si>
@@ -98,26 +98,62 @@
     <t>KARO</t>
   </si>
   <si>
-    <t>Kode Provinsi</t>
-  </si>
-  <si>
     <t>Nama Provinsi</t>
   </si>
   <si>
-    <t>Kode Kabupaten/Kota</t>
-  </si>
-  <si>
     <t>Nama Kabupaten/Kota</t>
   </si>
   <si>
     <t>Kode Peta (Map)</t>
+  </si>
+  <si>
+    <t>Kode Provinsi (BPS)</t>
+  </si>
+  <si>
+    <t>Kode Provinsi (DAPODIK)</t>
+  </si>
+  <si>
+    <t>Kode Kabupaten/Kota (BPS)</t>
+  </si>
+  <si>
+    <t>Kode Kabupaten/Kota (DAPODIK)</t>
+  </si>
+  <si>
+    <t>100000</t>
+  </si>
+  <si>
+    <t>100700</t>
+  </si>
+  <si>
+    <t>030000</t>
+  </si>
+  <si>
+    <t>032200</t>
+  </si>
+  <si>
+    <t>160000</t>
+  </si>
+  <si>
+    <t>160200</t>
+  </si>
+  <si>
+    <t>090000</t>
+  </si>
+  <si>
+    <t>096200</t>
+  </si>
+  <si>
+    <t>070000</t>
+  </si>
+  <si>
+    <t>070300</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,6 +168,10 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -151,15 +191,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{97583854-5DEC-4EBB-A287-0031D1824032}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -491,100 +536,158 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C16D64EC-EAF9-44BF-AF26-2506A6D457D2}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>